<commit_message>
마감 3배: 붕괴 240 / A 폐쇄 150 (ADR-0087)
ADR-0085가 잡은 붕괴 80 / A 폐쇄 50은 계약 왕복이 겨우 들어오는 값이었다.
A까지의 행동 예산이 중앙 38칸(표준세트 0.5회분)이라, 계약 하나를 끝내면
시설을 뒤질 칸이 남지 않았다. 구역 규모를 두 배로 키우는 변경과 함께
한 런에서 "무엇을 더 챙길까"를 고를 폭을 넓히려고 두 마감을 세 배로 늘린다.

RUN_COLLAPSE_TIME 80 -> 240, EXIT_A_DISABLED_AT 50 -> 150.
EXIT_OPEN_WINDOW(5), 가동 게이지(9~4칸), 작업 게이지, 증원 주기, 위협 이동
간격은 그대로다. 행동 예산은 중앙 138칸(표준세트 1.9회)이 되고, 아홉 계약
모두 전 시드에서 쓸 수 있는 출구를 갖는다.

코드에는 두 값을 하드코딩한 곳이 없어 상수만 바꿨다. 문서와 참조 엑셀,
ADR-0085의 상태(superseded)를 같은 변경에서 갱신한다.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/card-extraction-reference.xlsx
+++ b/docs/card-extraction-reference.xlsx
@@ -4006,7 +4006,7 @@
         <v>72</v>
       </c>
       <c r="C24" s="6">
-        <v>80</v>
+        <v>240</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>73</v>
@@ -4193,7 +4193,7 @@
         <v>105</v>
       </c>
       <c r="C35" s="5">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>106</v>
@@ -9019,7 +9019,7 @@
         <v>926</v>
       </c>
       <c r="C57" s="5">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="D57" s="5" t="s">
         <v>67</v>
@@ -9957,7 +9957,7 @@
         <v>1010</v>
       </c>
       <c r="C124" s="6">
-        <v>80</v>
+        <v>240</v>
       </c>
       <c r="D124" s="6" t="s">
         <v>67</v>

</xml_diff>